<commit_message>
Momentum scan results 2026-10-06
</commit_message>
<xml_diff>
--- a/results/momentum_2026-10-06.xlsx
+++ b/results/momentum_2026-10-06.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,198 +441,132 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>AEHR</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>FRSH</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SDEV</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RXRX</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MDLN</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ALAB</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>ASST</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>GTLB</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>FPS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>AXTI</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NVAX</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>COHR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>RXRX</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NTNX</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>PENG</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>MXL</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>TRMD</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>MU</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>PACB</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>XRPN</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>NBIS</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>SDGR</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>SKHY</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>

</xml_diff>